<commit_message>
QR Gen updated w. QRs
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="143">
   <si>
     <t>MERL-0003</t>
   </si>
@@ -84,6 +84,12 @@
   </si>
   <si>
     <t>TALHA AHMED</t>
+  </si>
+  <si>
+    <t>MERL-0069-06-SE</t>
+  </si>
+  <si>
+    <t>KINZA FATIMA</t>
   </si>
   <si>
     <t>MERL-0001</t>
@@ -844,6 +850,17 @@
         <v>23</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -863,18 +880,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
@@ -887,26 +904,26 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
@@ -919,34 +936,34 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12">
@@ -962,10 +979,10 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>6</v>
@@ -973,10 +990,10 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>6</v>
@@ -984,35 +1001,35 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18">
@@ -1028,35 +1045,35 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
@@ -1072,10 +1089,10 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>9</v>
@@ -1083,10 +1100,10 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>9</v>
@@ -1094,35 +1111,35 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
@@ -1160,10 +1177,10 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>14</v>
@@ -1171,10 +1188,10 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>17</v>
@@ -1193,10 +1210,10 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>9</v>
@@ -1204,50 +1221,50 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>14</v>
@@ -1255,50 +1272,50 @@
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>17</v>
@@ -1306,106 +1323,106 @@
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C59" s="5" t="s">
         <v>14</v>
@@ -1413,10 +1430,10 @@
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C60" s="5" t="s">
         <v>14</v>
@@ -1424,10 +1441,10 @@
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C61" s="5" t="s">
         <v>14</v>
@@ -1435,10 +1452,10 @@
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C62" s="5" t="s">
         <v>14</v>
@@ -1446,10 +1463,10 @@
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C63" s="5" t="s">
         <v>17</v>
@@ -1457,34 +1474,34 @@
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1"/>

</xml_diff>